<commit_message>
Change log -fixed context csv save timing -added % to split summary -changed holdout years to split each year in the holdout set in half, first half goes to val set, second goes to test set -made dataset years global vars -added best parameters return to bayes search. Saving dataframe -added model df, saving dataframe -removed temporary dataset split code (used for testing before I got henry code) -WIP implementing feature importance plotting
</commit_message>
<xml_diff>
--- a/ml/data/cre22_cleaning_report.xlsx
+++ b/ml/data/cre22_cleaning_report.xlsx
@@ -473,10 +473,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E2" t="n">
-        <v>10886</v>
+        <v>12667</v>
       </c>
     </row>
     <row r="3">
@@ -494,10 +494,10 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E3" t="n">
-        <v>44097</v>
+        <v>44111</v>
       </c>
     </row>
     <row r="4">
@@ -515,10 +515,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E4" t="n">
-        <v>3712</v>
+        <v>3786</v>
       </c>
     </row>
     <row r="5">
@@ -536,10 +536,10 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -557,7 +557,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E6" t="n">
         <v>12</v>
@@ -578,7 +578,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E7" t="n">
         <v>31</v>
@@ -599,7 +599,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E8" t="n">
         <v>4</v>
@@ -620,7 +620,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E9" t="n">
         <v>14</v>
@@ -641,10 +641,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E10" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11">
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E11" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12">
@@ -683,10 +683,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E12" t="n">
-        <v>87459</v>
+        <v>108512</v>
       </c>
     </row>
     <row r="13">
@@ -701,13 +701,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>155</v>
+        <v>201</v>
       </c>
       <c r="D13" t="n">
-        <v>103390</v>
+        <v>129528</v>
       </c>
       <c r="E13" t="n">
-        <v>2475</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -743,10 +743,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9815</v>
+        <v>11737</v>
       </c>
       <c r="D15" t="n">
-        <v>93730</v>
+        <v>117992</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -764,13 +764,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>513</v>
+        <v>593</v>
       </c>
       <c r="D16" t="n">
-        <v>103032</v>
+        <v>129136</v>
       </c>
       <c r="E16" t="n">
-        <v>13233</v>
+        <v>14989</v>
       </c>
     </row>
     <row r="17">
@@ -785,13 +785,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>8874</v>
+        <v>10832</v>
       </c>
       <c r="D17" t="n">
-        <v>94671</v>
+        <v>118897</v>
       </c>
       <c r="E17" t="n">
-        <v>230</v>
+        <v>246</v>
       </c>
     </row>
     <row r="18">
@@ -806,13 +806,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>8836</v>
+        <v>10772</v>
       </c>
       <c r="D18" t="n">
-        <v>94709</v>
+        <v>118957</v>
       </c>
       <c r="E18" t="n">
-        <v>75708</v>
+        <v>94164</v>
       </c>
     </row>
     <row r="19">
@@ -827,13 +827,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>8836</v>
+        <v>10771</v>
       </c>
       <c r="D19" t="n">
-        <v>94709</v>
+        <v>118958</v>
       </c>
       <c r="E19" t="n">
-        <v>75573</v>
+        <v>93964</v>
       </c>
     </row>
     <row r="20">
@@ -851,10 +851,10 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E20" t="n">
-        <v>37843</v>
+        <v>43280</v>
       </c>
     </row>
     <row r="21">
@@ -872,10 +872,10 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E21" t="n">
-        <v>77511</v>
+        <v>96456</v>
       </c>
     </row>
     <row r="22">
@@ -890,13 +890,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>47362</v>
+        <v>64218</v>
       </c>
       <c r="D22" t="n">
-        <v>56183</v>
+        <v>65511</v>
       </c>
       <c r="E22" t="n">
-        <v>297</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23">
@@ -911,13 +911,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>47729</v>
+        <v>64711</v>
       </c>
       <c r="D23" t="n">
-        <v>55816</v>
+        <v>65018</v>
       </c>
       <c r="E23" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24">
@@ -932,10 +932,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>47473</v>
+        <v>64366</v>
       </c>
       <c r="D24" t="n">
-        <v>56072</v>
+        <v>65363</v>
       </c>
       <c r="E24" t="n">
         <v>14</v>
@@ -953,13 +953,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>47548</v>
+        <v>64430</v>
       </c>
       <c r="D25" t="n">
-        <v>55997</v>
+        <v>65299</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26">
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>47357</v>
+        <v>64212</v>
       </c>
       <c r="D26" t="n">
-        <v>56188</v>
+        <v>65517</v>
       </c>
       <c r="E26" t="n">
-        <v>4455</v>
+        <v>4577</v>
       </c>
     </row>
     <row r="27">
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>47145</v>
+        <v>63956</v>
       </c>
       <c r="D27" t="n">
-        <v>56400</v>
+        <v>65773</v>
       </c>
       <c r="E27" t="n">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28">
@@ -1016,13 +1016,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>47145</v>
+        <v>63956</v>
       </c>
       <c r="D28" t="n">
-        <v>56400</v>
+        <v>65773</v>
       </c>
       <c r="E28" t="n">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29">
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E29" t="n">
         <v>18</v>
@@ -1061,10 +1061,10 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E30" t="n">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31">
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E31" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32">
@@ -1103,10 +1103,10 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E32" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33">
@@ -1121,10 +1121,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>63107</v>
+        <v>81668</v>
       </c>
       <c r="D33" t="n">
-        <v>40438</v>
+        <v>48061</v>
       </c>
       <c r="E33" t="n">
         <v>51</v>
@@ -1142,13 +1142,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>66902</v>
+        <v>85208</v>
       </c>
       <c r="D34" t="n">
-        <v>36643</v>
+        <v>44521</v>
       </c>
       <c r="E34" t="n">
-        <v>232</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35">
@@ -1166,10 +1166,10 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E35" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36">
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>48078</v>
+        <v>65016</v>
       </c>
       <c r="D36" t="n">
-        <v>55467</v>
+        <v>64713</v>
       </c>
       <c r="E36" t="n">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="37">
@@ -1205,13 +1205,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>47357</v>
+        <v>64212</v>
       </c>
       <c r="D37" t="n">
-        <v>56188</v>
+        <v>65517</v>
       </c>
       <c r="E37" t="n">
-        <v>4455</v>
+        <v>4577</v>
       </c>
     </row>
     <row r="38">
@@ -1229,10 +1229,10 @@
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E38" t="n">
-        <v>37843</v>
+        <v>43280</v>
       </c>
     </row>
     <row r="39">
@@ -1250,10 +1250,10 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
       <c r="E39" t="n">
-        <v>10886</v>
+        <v>12667</v>
       </c>
     </row>
   </sheetData>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>103557</v>
+        <v>129745</v>
       </c>
     </row>
     <row r="3">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103545</v>
+        <v>129729</v>
       </c>
     </row>
     <row r="4">
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B129"/>
+  <dimension ref="A1:B130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1401,7 +1401,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BETHLEHEM</t>
+          <t>BETHEL</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1411,7 +1411,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BLOOMFIELD</t>
+          <t>BETHLEHEM</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1421,7 +1421,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BOLTON</t>
+          <t>BLOOMFIELD</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1431,7 +1431,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BRANFORD</t>
+          <t>BOLTON</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1441,7 +1441,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BRIDGEPORT</t>
+          <t>BRANFORD</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1451,7 +1451,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BRISTOL</t>
+          <t>BRIDGEPORT</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1461,7 +1461,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BROOKFIELD</t>
+          <t>BRISTOL</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1471,7 +1471,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BROOKLYN</t>
+          <t>BROOKFIELD</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1481,7 +1481,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BURLINGTON</t>
+          <t>BROOKLYN</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1491,7 +1491,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CANTERBURY</t>
+          <t>BURLINGTON</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1501,7 +1501,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CANTON</t>
+          <t>CANTERBURY</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1511,7 +1511,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CHESHIRE</t>
+          <t>CANTON</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1521,7 +1521,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CHESTER</t>
+          <t>CHESHIRE</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1531,7 +1531,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CLINTON</t>
+          <t>CHESTER</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1541,7 +1541,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CORNWALL</t>
+          <t>CLINTON</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1551,7 +1551,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>COVENTRY</t>
+          <t>CORNWALL</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1561,7 +1561,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CROMWELL</t>
+          <t>COVENTRY</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1571,7 +1571,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DANBURY</t>
+          <t>CROMWELL</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1581,7 +1581,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DARIEN</t>
+          <t>DANBURY</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1591,7 +1591,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DEEP RIVER</t>
+          <t>DARIEN</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1601,7 +1601,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DERBY</t>
+          <t>DEEP RIVER</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1611,7 +1611,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DURHAM</t>
+          <t>DERBY</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1621,7 +1621,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>EAST HADDAM</t>
+          <t>DURHAM</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1631,7 +1631,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EAST HAMPTON</t>
+          <t>EAST HADDAM</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1641,7 +1641,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>EAST HARTFORD</t>
+          <t>EAST HAMPTON</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1651,7 +1651,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EAST HAVEN</t>
+          <t>EAST HARTFORD</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1661,7 +1661,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>EAST LYME</t>
+          <t>EAST HAVEN</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1671,7 +1671,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>EASTFORD</t>
+          <t>EAST LYME</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1681,7 +1681,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>EASTON</t>
+          <t>EASTFORD</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1691,7 +1691,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ENFIELD</t>
+          <t>EASTON</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1701,7 +1701,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FAIRFIELD</t>
+          <t>ENFIELD</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1711,7 +1711,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FARMINGTON</t>
+          <t>FAIRFIELD</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1721,7 +1721,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GLASTONBURY</t>
+          <t>FARMINGTON</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1731,7 +1731,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GOSHEN</t>
+          <t>GLASTONBURY</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1741,7 +1741,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GRANBY</t>
+          <t>GOSHEN</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1751,7 +1751,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GREENWICH</t>
+          <t>GRANBY</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1761,7 +1761,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GROTON</t>
+          <t>GREENWICH</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1771,7 +1771,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GUILFORD</t>
+          <t>GROTON</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1781,7 +1781,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>HADDAM</t>
+          <t>GUILFORD</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1791,7 +1791,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>HAMDEN</t>
+          <t>HADDAM</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1801,7 +1801,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>HAMPTON</t>
+          <t>HAMDEN</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1811,7 +1811,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HARTFORD</t>
+          <t>HAMPTON</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1821,7 +1821,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>HARWINTON</t>
+          <t>HARTFORD</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1831,7 +1831,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>KILLINGLY</t>
+          <t>HARWINTON</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1841,7 +1841,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>KILLINGWORTH</t>
+          <t>KILLINGLY</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1851,7 +1851,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LEBANON</t>
+          <t>KILLINGWORTH</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1861,7 +1861,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LEDYARD</t>
+          <t>LEBANON</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1871,7 +1871,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LITCHFIELD</t>
+          <t>LEDYARD</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1881,7 +1881,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LYME</t>
+          <t>LITCHFIELD</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1891,7 +1891,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MADISON</t>
+          <t>LYME</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1901,7 +1901,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MANCHESTER</t>
+          <t>MADISON</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1911,7 +1911,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MANSFIELD</t>
+          <t>MANCHESTER</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1921,7 +1921,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MARLBOROUGH</t>
+          <t>MANSFIELD</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1931,7 +1931,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MERIDEN</t>
+          <t>MARLBOROUGH</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1941,7 +1941,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MIDDLEBURY</t>
+          <t>MERIDEN</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1951,7 +1951,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MIDDLETOWN</t>
+          <t>MIDDLEBURY</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1961,7 +1961,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MILFORD</t>
+          <t>MIDDLETOWN</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1971,7 +1971,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MONROE</t>
+          <t>MILFORD</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1981,7 +1981,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MONTVILLE</t>
+          <t>MONROE</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1991,7 +1991,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MORRIS</t>
+          <t>MONTVILLE</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2001,7 +2001,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>NAUGATUCK</t>
+          <t>MORRIS</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2011,7 +2011,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>NEW BRITAIN</t>
+          <t>NAUGATUCK</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2021,7 +2021,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NEW CANAAN</t>
+          <t>NEW BRITAIN</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2031,7 +2031,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NEW FAIRFIELD</t>
+          <t>NEW CANAAN</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2041,7 +2041,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NEW HARTFORD</t>
+          <t>NEW FAIRFIELD</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2051,7 +2051,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>NEW HAVEN</t>
+          <t>NEW HARTFORD</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2061,7 +2061,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>NEW LONDON</t>
+          <t>NEW HAVEN</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2071,7 +2071,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>NEW MILFORD</t>
+          <t>NEW LONDON</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2081,7 +2081,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NEWINGTON</t>
+          <t>NEW MILFORD</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2091,7 +2091,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>NEWTOWN</t>
+          <t>NEWINGTON</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2101,7 +2101,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NORFOLK</t>
+          <t>NEWTOWN</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2111,7 +2111,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>NORTH CANAAN</t>
+          <t>NORFOLK</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2121,7 +2121,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NORTH HAVEN</t>
+          <t>NORTH CANAAN</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2131,7 +2131,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>NORWICH</t>
+          <t>NORTH HAVEN</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2141,7 +2141,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>OLD LYME</t>
+          <t>NORWICH</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2151,7 +2151,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>OLD SAYBROOK</t>
+          <t>OLD LYME</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2161,7 +2161,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ORANGE</t>
+          <t>OLD SAYBROOK</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2171,7 +2171,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PLAINFIELD</t>
+          <t>ORANGE</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2181,7 +2181,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PLAINVILLE</t>
+          <t>PLAINFIELD</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2191,7 +2191,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PLYMOUTH</t>
+          <t>PLAINVILLE</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2201,7 +2201,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PORTLAND</t>
+          <t>PLYMOUTH</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2211,7 +2211,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PRESTON</t>
+          <t>PORTLAND</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2221,7 +2221,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PROSPECT</t>
+          <t>PRESTON</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2231,7 +2231,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>REDDING</t>
+          <t>PROSPECT</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2241,7 +2241,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RIDGEFIELD</t>
+          <t>REDDING</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2251,7 +2251,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ROCKY HILL</t>
+          <t>RIDGEFIELD</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2261,7 +2261,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SALEM</t>
+          <t>ROCKY HILL</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2271,7 +2271,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SALISBURY</t>
+          <t>SALEM</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2281,7 +2281,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SCOTLAND</t>
+          <t>SALISBURY</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2291,7 +2291,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SEYMOUR</t>
+          <t>SCOTLAND</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2301,7 +2301,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SHARON</t>
+          <t>SEYMOUR</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2311,7 +2311,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SHELTON</t>
+          <t>SHARON</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2321,7 +2321,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SIMSBURY</t>
+          <t>SHELTON</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2331,7 +2331,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SOUTH WINDSOR</t>
+          <t>SIMSBURY</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2341,7 +2341,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SOUTHBURY</t>
+          <t>SOUTH WINDSOR</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2351,7 +2351,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SOUTHINGTON</t>
+          <t>SOUTHBURY</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2361,7 +2361,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SPRAGUE</t>
+          <t>SOUTHINGTON</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2371,7 +2371,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>STERLING</t>
+          <t>SPRAGUE</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2381,7 +2381,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>STONINGTON</t>
+          <t>STERLING</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2391,7 +2391,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>STRATFORD</t>
+          <t>STONINGTON</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2401,7 +2401,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SUFFIELD</t>
+          <t>STRATFORD</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2411,7 +2411,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>TOLLAND</t>
+          <t>SUFFIELD</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2421,7 +2421,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>TORRINGTON</t>
+          <t>TOLLAND</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2431,7 +2431,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TRUMBULL</t>
+          <t>TORRINGTON</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2441,7 +2441,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>UNION</t>
+          <t>TRUMBULL</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2451,7 +2451,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>VOLUNTOWN</t>
+          <t>UNION</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2461,7 +2461,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>WALLINGFORD</t>
+          <t>VOLUNTOWN</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2471,7 +2471,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>WARREN</t>
+          <t>WALLINGFORD</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2481,7 +2481,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>WATERBURY</t>
+          <t>WARREN</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2491,7 +2491,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>WATERTOWN</t>
+          <t>WATERBURY</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2501,7 +2501,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>WEST HAVEN</t>
+          <t>WATERTOWN</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2511,7 +2511,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>WESTON</t>
+          <t>WEST HAVEN</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2521,7 +2521,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>WESTPORT</t>
+          <t>WESTON</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2531,7 +2531,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>WETHERSFIELD</t>
+          <t>WESTPORT</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2541,7 +2541,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>WILLINGTON</t>
+          <t>WETHERSFIELD</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2551,7 +2551,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>WILTON</t>
+          <t>WILLINGTON</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2561,7 +2561,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>WINCHESTER</t>
+          <t>WILTON</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2571,7 +2571,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>WINDSOR</t>
+          <t>WINCHESTER</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2581,7 +2581,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>WINDSOR LOCKS</t>
+          <t>WINDSOR</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2591,7 +2591,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>WOLCOTT</t>
+          <t>WINDSOR LOCKS</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2601,7 +2601,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>WOODBRIDGE</t>
+          <t>WOLCOTT</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2611,11 +2611,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>WOODBURY</t>
+          <t>WOODBRIDGE</t>
         </is>
       </c>
       <c r="B129" t="n">
         <v>128</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>WOODBURY</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2629,7 +2639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B137"/>
+  <dimension ref="A1:B147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2667,7 +2677,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3 FAMILY</t>
+          <t>3 FAM</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2677,7 +2687,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3-4 FAMILY</t>
+          <t>3 FAMILY</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2687,7 +2697,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4 FAMILY</t>
+          <t>3-4 FAMILY</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2697,7 +2707,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>55+ UNIT</t>
+          <t>4 FAM</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2707,7 +2717,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ANTIQUE</t>
+          <t>4 FAMILY</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2717,7 +2727,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>APART COMPLEX</t>
+          <t>55+ UNIT</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2727,7 +2737,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>APARTMENTS</t>
+          <t>ANTIQUE</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2737,7 +2747,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>APARTMENTS NEWER</t>
+          <t>APART COMPLEX</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2747,7 +2757,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>APT-STUDIO/BARN</t>
+          <t>APARTMENT RES/COM</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2757,7 +2767,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>APT/GARAGE</t>
+          <t>APARTMENTS</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2767,7 +2777,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>APT/RES GARAGE</t>
+          <t>APARTMENTS NEWER</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2777,7 +2787,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ASSISTED LIVING</t>
+          <t>APT-STUDIO/BARN</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2787,7 +2797,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AUTO SHOWROOM</t>
+          <t>APT/GARAGE</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2797,7 +2807,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BARN HOUSE</t>
+          <t>APT/RES GARAGE</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2807,7 +2817,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BEACH CONDO</t>
+          <t>ASSISTED LIVING</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2817,7 +2827,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BEACH CONTEMP</t>
+          <t>AUTO SHOWROOM</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2827,7 +2837,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BRANCH BANK</t>
+          <t>BARN HOUSE</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2837,7 +2847,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BUNGALOW</t>
+          <t>BEACH CONDO</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2847,7 +2857,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CABANA</t>
+          <t>BEACH CONTEMP</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2857,7 +2867,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAMP</t>
+          <t>BRANCH BANK</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2867,7 +2877,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAPE</t>
+          <t>BUNGALOW</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2877,7 +2887,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAPE COD</t>
+          <t>CABANA</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2887,7 +2897,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAPE PAD</t>
+          <t>CAMP</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2897,7 +2907,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAR DEALER</t>
+          <t>CAPE</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2907,7 +2917,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CENTURY+</t>
+          <t>CAPE COD</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2917,7 +2927,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CHURCHES</t>
+          <t>CAPE PAD</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2927,7 +2937,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CLUBS/LODGES</t>
+          <t>CAR DEALER</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2937,7 +2947,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>COLONIAL</t>
+          <t>CAR WASH</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2947,7 +2957,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>COLONIAL (COVE)</t>
+          <t>CENTURY+</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2957,7 +2967,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>COLONIAL EXPANDED</t>
+          <t>CHURCHES</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2967,7 +2977,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>COLONIAL MODERN</t>
+          <t>CLUBS/LODGES</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2977,7 +2987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>COLONIAL PAD</t>
+          <t>COLONIAL</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2987,7 +2997,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>COLONIAL S</t>
+          <t>COLONIAL (COVE)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2997,7 +3007,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>COMM STYLE RES</t>
+          <t>COLONIAL EXPANDED</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3007,7 +3017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>COMMERCIAL</t>
+          <t>COLONIAL MODERN</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -3017,7 +3027,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CONDO CAPE</t>
+          <t>COLONIAL PAD</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3027,7 +3037,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CONDO COLONIAL</t>
+          <t>COLONIAL S</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3037,7 +3047,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CONDO RANCH</t>
+          <t>COMM STYLE RES</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3047,7 +3057,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CONDO TOWNHOUSE</t>
+          <t>COMMERCIAL</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -3057,7 +3067,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CONDO UNIT</t>
+          <t>CONDO CAPE</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3067,7 +3077,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CONDOMINIUM</t>
+          <t>CONDO COLONIAL</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -3077,7 +3087,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CONTEMPORARY</t>
+          <t>CONDO RANCH</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -3087,7 +3097,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CONV/S S GAS</t>
+          <t>CONDO TOWNHOUSE</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3097,7 +3107,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CONVENTIONAL</t>
+          <t>CONDO UNIT</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -3107,7 +3117,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>COTTAGE</t>
+          <t>CONDOMINIUM</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -3117,7 +3127,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>COTTAGE (COVE)</t>
+          <t>CONGREGATE LIVING</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -3127,7 +3137,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CRAFTSMAN CAPE</t>
+          <t>CONTEMPORARY</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -3137,7 +3147,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>CONV/S S GAS</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -3147,7 +3157,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CUSTOM COLONIAL</t>
+          <t>CONVENTIONAL</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -3157,7 +3167,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CUSTOM CONTEMPORARY</t>
+          <t>COTTAGE</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -3167,7 +3177,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CUSTOM DESIGN</t>
+          <t>COTTAGE (COVE)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -3177,7 +3187,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DAYCARE</t>
+          <t>CRAFTSMAN CAPE</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -3187,7 +3197,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DUPLEX</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -3197,7 +3207,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DUPLEX/TRIPLEX</t>
+          <t>CUSTOM COLONIAL</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -3207,7 +3217,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DUTCH COLONIAL</t>
+          <t>CUSTOM CONTEMPORARY</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -3217,7 +3227,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DW MOBILE HOME</t>
+          <t>CUSTOM DESIGN</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3227,7 +3237,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ESTATE</t>
+          <t>DAYCARE</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -3237,7 +3247,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>FAMILY CONVER.</t>
+          <t>DUPLEX</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3247,7 +3257,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FAMILY DUPLEX</t>
+          <t>DUPLEX/TRIPLEX</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -3257,7 +3267,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>FAMILY FLAT</t>
+          <t>DUTCH COLONIAL</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3267,7 +3277,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>FEDERALIST</t>
+          <t>DW MOBILE HOME</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -3277,7 +3287,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FOUR FAMILY</t>
+          <t>ESTATE</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3287,7 +3297,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GAR/APARTMENT</t>
+          <t>FAMILY CONVER.</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -3297,7 +3307,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GARAGE/LIV SPACE</t>
+          <t>FAMILY DUPLEX</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3307,7 +3317,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GARAGE/OFFICE</t>
+          <t>FAMILY FLAT</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -3317,7 +3327,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>HALF DUPLEX</t>
+          <t>FEDERALIST</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3327,7 +3337,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>HIGH RANCH</t>
+          <t>FOUR FAMILY</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -3337,7 +3347,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HISTORIC HOME</t>
+          <t>GAR/APARTMENT</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3347,7 +3357,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>HISTORICAL HSE</t>
+          <t>GARAGE/LIV SPACE</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -3357,7 +3367,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>JOB SHOP(S)</t>
+          <t>GARAGE/OFFICE</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3367,7 +3377,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LIGHT INDUSTRIAL</t>
+          <t>HALF DUPLEX</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -3377,7 +3387,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LOG CABIN</t>
+          <t>HIGH RANCH</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3387,7 +3397,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MANUFACTURED HOME</t>
+          <t>HISTORIC HOME</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -3397,7 +3407,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MED. OFFICE</t>
+          <t>HISTORICAL HSE</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3407,7 +3417,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MEDICAL OFFICE</t>
+          <t>INN</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -3417,7 +3427,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MFG DWELL</t>
+          <t>JOB SHOP(S)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3427,7 +3437,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MINI MART</t>
+          <t>LIGHT INDUSTRIAL</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -3437,7 +3447,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>MOBILE HOME</t>
+          <t>LOG CABIN</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -3447,7 +3457,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MODERN COLONIAL</t>
+          <t>MANUFACTURED HOME</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -3457,7 +3467,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MODERN/CONTEMP</t>
+          <t>MED. OFFICE</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -3467,7 +3477,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MULTI FAMILY</t>
+          <t>MEDICAL OFFICE</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -3477,7 +3487,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MULTI-FAMILY</t>
+          <t>MFG DWELL</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -3487,7 +3497,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>NEW CONVENTIONAL</t>
+          <t>MINI MART</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -3497,7 +3507,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>OFF-STUDIO/RES GAR</t>
+          <t>MOBILE HOME</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -3507,7 +3517,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>OFFICE</t>
+          <t>MODERN COLONIAL</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -3517,7 +3527,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>OFFICE BLDG</t>
+          <t>MODERN/CONTEMP</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -3527,7 +3537,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>OFFICE/APARTMENTS</t>
+          <t>MULTI FAMILY</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -3537,7 +3547,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>OFFICE/APT</t>
+          <t>MULTI-FAMILY</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -3547,7 +3557,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>OFFICE/APT COM</t>
+          <t>NEW CONVENTIONAL</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -3557,7 +3567,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>OFFICE/RES TYP</t>
+          <t>OFF-STUDIO/RES GAR</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -3567,7 +3577,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>OFFICE/RETAIL</t>
+          <t>OFFICE</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -3577,7 +3587,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>OLD STYLE</t>
+          <t>OFFICE BLDG</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -3587,7 +3597,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>OLD STYLE APT</t>
+          <t>OFFICE CONDO</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -3597,7 +3607,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>OUTBUILDINGS</t>
+          <t>OFFICE/APARTMENTS</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -3607,7 +3617,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>POOL HSE</t>
+          <t>OFFICE/APT</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -3617,7 +3627,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PRE-ENG MFG</t>
+          <t>OFFICE/APT COM</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -3627,7 +3637,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>RAISED CAPE</t>
+          <t>OFFICE/RES TYP</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -3637,7 +3647,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>RAISED RANCH</t>
+          <t>OFFICE/RETAIL</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -3647,7 +3657,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>RANCH</t>
+          <t>OLD STYLE</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -3657,7 +3667,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>RES APT HSE</t>
+          <t>OLD STYLE APT</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -3667,7 +3677,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>RES CONDO</t>
+          <t>OUTBLDGS</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -3677,7 +3687,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>RES CONVERSION</t>
+          <t>OUTBUILDINGS</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -3687,7 +3697,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>RES STYLE COMM</t>
+          <t>POOL HSE</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -3697,7 +3707,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>RES STYLE OFF/MIXED</t>
+          <t>PRE-ENG MFG</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -3707,7 +3717,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>RES TYP COM</t>
+          <t>RAISED CAPE</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -3717,7 +3727,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>RES TYPE COM</t>
+          <t>RAISED RANCH</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -3727,7 +3737,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>RETAIL STRIP STORES</t>
+          <t>RANCH</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -3737,7 +3747,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>RETAIL/APT</t>
+          <t>RES APT HSE</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -3747,7 +3757,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>RETAIL/OFFICE MIX</t>
+          <t>RES CONDO</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -3757,7 +3767,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ROOMING HOUSE</t>
+          <t>RES CONVERSION</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -3767,7 +3777,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ROOMNG/ BOARDNG HSE</t>
+          <t>RES STYLE COMM</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -3777,7 +3787,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ROW HOUSE</t>
+          <t>RES STYLE OFF/MIXED</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -3787,7 +3797,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SCHOOLS-PUBLIC</t>
+          <t>RES TP COMM</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -3797,7 +3807,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SERVICE SHOP</t>
+          <t>RES TYP COM</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -3807,7 +3817,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SF W/INLAW</t>
+          <t>RES TYPE COM</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -3817,7 +3827,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SNGL FAM ATTAC</t>
+          <t>RESTAURANT</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -3827,7 +3837,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SPLIT LEVEL</t>
+          <t>RETAIL STRIP STORES</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -3837,7 +3847,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SPLIT-LEVEL</t>
+          <t>RETAIL/APT</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -3847,7 +3857,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>STORE</t>
+          <t>RETAIL/OFFICE MIX</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -3857,7 +3867,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>STORES/APT</t>
+          <t>ROOMING HOUSE</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -3867,7 +3877,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>STORES/APT COM</t>
+          <t>ROOMNG/ BOARDNG HSE</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -3877,7 +3887,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>STUDIO</t>
+          <t>ROW HOUSE</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -3887,7 +3897,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>STUDIO/HM OFFICE</t>
+          <t>SCHOOLS-PUBLIC</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -3897,7 +3907,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>THREE FAMILY</t>
+          <t>SERVICE SHOP</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -3907,7 +3917,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TOWNHOUSE</t>
+          <t>SF W/INLAW</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -3917,7 +3927,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>TRADITIONAL</t>
+          <t>SNGL FAM ATTAC</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -3927,7 +3937,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>TUDOR</t>
+          <t>SPLIT LEVEL</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -3937,7 +3947,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>TWO FAMILY</t>
+          <t>SPLIT-LEVEL</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -3947,7 +3957,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>VACANT</t>
+          <t>STORE</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -3957,7 +3967,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>VACANT LAND</t>
+          <t>STORES/APT</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -3967,7 +3977,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>VCAANT</t>
+          <t>STORES/APT COM</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -3977,7 +3987,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>VICTORIAN</t>
+          <t>STUDIO</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -3987,7 +3997,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>WAREHOUSE</t>
+          <t>STUDIO/HM OFFICE</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -3997,11 +4007,111 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>WATER PLANT</t>
+          <t>THREE FAMILY</t>
         </is>
       </c>
       <c r="B137" t="n">
         <v>136</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>TOWNHOUSE</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>TRADITIONAL</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>TUDOR</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>TWO FAMILY</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>VACANT</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>VACANT LAND</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>VCAANT</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>VICTORIAN</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>WAREHOUSE</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>WATER PLANT</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>